<commit_message>
Auto update Pengadaan 2026-10-25 10:09:02
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-25).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-25).xlsx
@@ -1567,22 +1567,22 @@
         <v>283157746</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>30118025</v>
+        <v>50235125</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>26778260</v>
+        <v>46526860</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>253039721</v>
+        <v>232922621</v>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
@@ -1867,28 +1867,28 @@
         </is>
       </c>
       <c r="C40" s="7" t="n">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="D40" s="9" t="n">
         <v>956575994</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>750435556</v>
+        <v>783150756</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>652591561</v>
+        <v>685306761</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>206140438</v>
+        <v>173425238</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -3325,28 +3325,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4067</v>
+        <v>4058</v>
       </c>
       <c r="D77" s="13" t="n">
         <v>34392291062</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>562</v>
+        <v>580</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>7334150952</v>
+        <v>7386983252</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>562</v>
+        <v>580</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>20088396779.6</v>
+        <v>20140860579.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3505</v>
+        <v>3478</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27058140110</v>
+        <v>27005307810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>